<commit_message>
Added new RDF data schemes and visual schemes for environment-table17-18, and fixed XLSX spreadsheets for environment-table17-18
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/environment-table17.xlsx
+++ b/sources/table_normalization/xlsx/environment-table17.xlsx
@@ -495,7 +495,6 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -512,7 +511,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
@@ -525,6 +523,8 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -832,7 +832,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1053,36 +1053,36 @@
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33"/>
-      <c r="I2" s="34" t="s">
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="33" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="26.15" customHeight="1">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="42"/>
-      <c r="D3" s="42"/>
-      <c r="E3" s="42"/>
-      <c r="F3" s="42"/>
-      <c r="G3" s="42"/>
-      <c r="H3" s="42"/>
-      <c r="I3" s="43" t="s">
+      <c r="C3" s="40"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="40"/>
+      <c r="G3" s="40"/>
+      <c r="H3" s="40"/>
+      <c r="I3" s="41" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="130.5" customHeight="1">
-      <c r="A4" s="40"/>
+      <c r="A4" s="43"/>
       <c r="B4" s="4" t="s">
         <v>6</v>
       </c>
@@ -1104,7 +1104,7 @@
       <c r="H4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="I4" s="44"/>
+      <c r="I4" s="42"/>
       <c r="J4" s="5"/>
     </row>
     <row r="5" spans="1:12" ht="24.9" customHeight="1">
@@ -1549,7 +1549,7 @@
       </c>
     </row>
     <row r="19" spans="1:12" ht="24.9" customHeight="1">
-      <c r="A19" s="36" t="s">
+      <c r="A19" s="35" t="s">
         <v>29</v>
       </c>
       <c r="B19" s="21">
@@ -1597,7 +1597,7 @@
       </c>
     </row>
     <row r="20" spans="1:12" ht="24.9" customHeight="1">
-      <c r="A20" s="37" t="s">
+      <c r="A20" s="36" t="s">
         <v>31</v>
       </c>
       <c r="B20" s="24">
@@ -1634,7 +1634,7 @@
       </c>
     </row>
     <row r="21" spans="1:12" ht="24.9" customHeight="1">
-      <c r="A21" s="37" t="s">
+      <c r="A21" s="36" t="s">
         <v>32</v>
       </c>
       <c r="B21" s="25">
@@ -1671,7 +1671,7 @@
       </c>
     </row>
     <row r="22" spans="1:12" ht="24.9" customHeight="1">
-      <c r="A22" s="37" t="s">
+      <c r="A22" s="36" t="s">
         <v>33</v>
       </c>
       <c r="B22" s="26">
@@ -1708,7 +1708,7 @@
       </c>
     </row>
     <row r="23" spans="1:12" ht="24.9" customHeight="1">
-      <c r="A23" s="38" t="s">
+      <c r="A23" s="37" t="s">
         <v>34</v>
       </c>
       <c r="B23" s="28">
@@ -1738,7 +1738,7 @@
       <c r="J23" s="1"/>
     </row>
     <row r="24" spans="1:12" ht="24.9" customHeight="1">
-      <c r="A24" s="35" t="s">
+      <c r="A24" s="34" t="s">
         <v>35</v>
       </c>
       <c r="B24" s="29"/>

</xml_diff>